<commit_message>
QA: apply confirmed rules (ADK = Adult Kit, gift pack noindex intentional, commemorative prints)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-09-26/qa_2026-09-26.xlsx
+++ b/listing-monitor/reports/2026-09-26/qa_2026-09-26.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-09-26 22:26. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-09-27 08:29. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3073,108 +3073,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SKU ADK</t>
+          <t>Short sleeve</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>SOP ghi ADK = combo Adult + Kid, nhưng trên web ADK đang dùng cho Adult Kit (áo + quần người lớn). Tool đang hiểu ADK = Adult. Đúng không?</t>
+          <t>SOP: không bao giờ nhắc short sleeve. Description KFK (130/162 listing), RFK (107/289), CFS (6) đang có 'Short-Sleeve shirt' / 'short sleeves'. Có cần xoá không?</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Short sleeve</t>
+          <t>Trustpilot / 4.9★</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>SOP: không bao giờ nhắc short sleeve. Nhưng template description KFK có 'Short-Sleeve shirt' và 'Sleeve length: Short sleeve'. Có cần xoá khỏi template không?</t>
+          <t>SOP: tránh 'Trustpilot' và claim 4.9★. Short description KFK, RFS, RFK có dòng 'Rated 4.9 on Trustpilot' (CFS không có). Giữ hay bỏ?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trustpilot / 4.9★</t>
+          <t>Tên né thương hiệu</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>SOP: tránh 'Trustpilot' và claim 4.9★. Short description KFK và một số meta đang dùng. Đây là template được duyệt hay cần sửa?</t>
+          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG và nhận ra kiểu 'Arsn@l', 'Lvr^_^pooI'.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tên né thương hiệu</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG. Còn tên thay thế nào khác không?</t>
+          <t>Tool KHÔNG báo lỗi 'sleeve badge' (tên option), chỉ báo 'badge' đứng riêng.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WINNERS / CHAMPIONS</t>
+          <t>Độ dài SEO title</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Listing in chữ kỷ niệm (vd 'CHAMPIONS 26') không bị báo thiếu player attribute/category. Đúng không?</t>
+          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gift pack NOINDEX</t>
+          <t>KFK / CFS / RFK template SEO</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Một số gift pack KFK (Bay^_^rn, P^_^SG) đang để noindex. Cố ý (né thương hiệu) hay lỗi?</t>
+          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Đã xác nhận 27/9</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Tool KHÔNG báo lỗi 'sleeve badge' (tên option), chỉ báo 'badge' đứng riêng. Đúng không?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Độ dài SEO title</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>KFK / CFS / RFK template SEO</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
+          <t>ADK = Adult Kit. Gift pack noindex là cố ý (không báo lỗi). Listing in 'CHAMPIONS 26 / WINNERS 26' không cần player attribute.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QA: short sleeve mention is fine, flag only sleeve mismatches
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-09-26/qa_2026-09-26.xlsx
+++ b/listing-monitor/reports/2026-09-26/qa_2026-09-26.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Cần xác nhận" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lỗi chi tiết'!$A$1:$M$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lỗi chi tiết'!$A$1:$M$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-09-27 08:29. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-09-27 08:38. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -658,118 +658,99 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sleeve</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Lỗi</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Số listing</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>SEO</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" t="n">
-        <v>13</v>
-      </c>
-      <c r="E14" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Lỗi lặp lại trên phần lớn listing của 1 site (nhiều khả năng do TEMPLATE, sửa template 1 lần)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Nhóm</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Vị trí</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Lỗi</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Số listing</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CFS</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Meta description</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>khoảng trắng trước dấu câu</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>9/13</t>
         </is>
@@ -786,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -963,22 +944,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sleeve</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Short description</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Có nhắc 'short sleeve' (quy tắc: không bao giờ nhắc short sleeve): ...ith no name or number applied. It includes a Short-Sleeve shirt, matching shorts and matching socks. P...</t>
+          <t>'Trustpilot' (...tomers ⭐ Rated 4.9/5 ★★★★★ on Trustpilot 🎁 Premium Kids Kits &amp; Gift Sp...)</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Xoá cụm 'short sleeve'</t>
+          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -1006,20 +987,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-26 14:09</t>
+          <t>2026-09-26 14:12</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>249870</v>
+        <v>249883</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>KFK_Redtrophy_HO_ADK_No_26/27</t>
+          <t>KFK_Redtrophy_AW_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Lvr^_^pooI Home Adult Football Kit 2026/27 (With socks)</t>
+          <t>Lvr^_^pooI Away Adult Football Kit 2026/27 (With socks)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1045,7 +1026,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/l-p-home-adult-football-kit-2026-27/</t>
+          <t>https://kidsfootballkit.co.uk/product/l-p-away-adult-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
@@ -1062,30 +1043,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KFK</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-09-26 14:12</t>
-        </is>
-      </c>
+          <t>RFS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>249883</v>
+        <v>103706</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>KFK_Redtrophy_AW_ADK_No_26/27</t>
+          <t>RFS_RM_AW_KD_No_26/27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Lvr^_^pooI Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sleeve</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1095,18 +1072,18 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Có nhắc 'short sleeve' (quy tắc: không bao giờ nhắc short sleeve): ...dult Football Kit 2026/27 is supplied with a Short-Sleeve shirt, matching shorts and matching socks. I...</t>
+          <t>'sponsor' (...ripes, collar trim, and front sponsor logos stand out sharply again...); 'worldwide' (...rid continues to inspire fans worldwide with its philosophy of ambiti...)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Xoá cụm 'short sleeve'</t>
+          <t>sponsor -&gt; front graphic / sleeve detail; worldwide -&gt; (bỏ)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/l-p-away-adult-football-kit-2026-27/</t>
+          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -1123,25 +1100,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KFK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-09-26 14:12</t>
-        </is>
-      </c>
+          <t>RFS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>249883</v>
+        <v>103706</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>KFK_Redtrophy_AW_ADK_No_26/27</t>
+          <t>RFS_RM_AW_KD_No_26/27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Lvr^_^pooI Away Adult Football Kit 2026/27 (With socks)</t>
+          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1156,7 +1129,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (...tomers ⭐ Rated 4.9/5 ★★★★★ on Trustpilot 🎁 Premium Kids Kits &amp; Gift Sp...)</t>
+          <t>'Trustpilot' (★ Rated 4.9 on Trustpilot By 100+ customers ✈ Fully Tra...)</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -1167,7 +1140,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/l-p-away-adult-football-kit-2026-27/</t>
+          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1187,18 +1160,22 @@
           <t>RFS</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-09-26 08:53</t>
+        </is>
+      </c>
       <c r="D7" t="n">
-        <v>103706</v>
+        <v>104055</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>RFS_RM_AW_KD_No_26/27</t>
+          <t>RFS_AH_HO_AD_No_26/27</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
+          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1213,18 +1190,18 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>'sponsor' (...ripes, collar trim, and front sponsor logos stand out sharply again...); 'worldwide' (...rid continues to inspire fans worldwide with its philosophy of ambiti...)</t>
+          <t>'official' (...r and sleeve cuffs, featuring official sponsor logos including “NHC”...); 'sponsor' (...eve cuffs, featuring official sponsor logos including “NHC” on the ...); 'features the' (...husiasts. This replica jersey features the club’s iconic royal blue base...); 'worldwide' (...nate local community and fans worldwide. Known as “Al-Za’eem,” the te...)</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>sponsor -&gt; front graphic / sleeve detail; worldwide -&gt; (bỏ)</t>
+          <t>official -&gt; football-inspired; sponsor -&gt; front graphic / sleeve detail; features the -&gt; includes the / highlights the; worldwide -&gt; (bỏ)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
+          <t>https://replicafootballshirt.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
@@ -1244,18 +1221,22 @@
           <t>RFS</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-09-26 08:53</t>
+        </is>
+      </c>
       <c r="D8" t="n">
-        <v>103706</v>
+        <v>104055</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>RFS_RM_AW_KD_No_26/27</t>
+          <t>RFS_AH_HO_AD_No_26/27</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
+          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1281,7 +1262,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
+          <t>https://replicafootballshirt.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -1291,9 +1272,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1301,48 +1282,44 @@
           <t>RFS</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-09-26 08:53</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>104055</v>
+        <v>103706</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>RFS_AH_HO_AD_No_26/27</t>
+          <t>RFS_RM_AW_KD_No_26/27</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
+          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>'official' (...r and sleeve cuffs, featuring official sponsor logos including “NHC”...); 'sponsor' (...eve cuffs, featuring official sponsor logos including “NHC” on the ...); 'features the' (...husiasts. This replica jersey features the club’s iconic royal blue base...); 'worldwide' (...nate local community and fans worldwide. Known as “Al-Za’eem,” the te...)</t>
+          <t>SEO title dài 69 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>official -&gt; football-inspired; sponsor -&gt; front graphic / sleeve detail; features the -&gt; includes the / highlights the; worldwide -&gt; (bỏ)</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://replicafootballshirt.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
+          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
@@ -1352,9 +1329,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1382,22 +1359,22 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>'Trustpilot' (★ Rated 4.9 on Trustpilot By 100+ customers ✈ Fully Tra...)</t>
+          <t>SEO title dài 68 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Trustpilot -&gt; (bỏ claim không kiểm chứng)</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -1420,21 +1397,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RFS</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-09-26 01:30</t>
+        </is>
+      </c>
       <c r="D11" t="n">
-        <v>103706</v>
+        <v>81726</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>RFS_RM_AW_KD_No_26/27</t>
+          <t>CFS_NC_GreyGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Real Madrid Away Kid Replica Football Kit 2026/27</t>
+          <t>Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1444,12 +1425,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 69 ký tự (nên &lt;= 60)</t>
+          <t>Meta dài 180 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1460,7 +1441,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://replicafootballshirt.com/product/real-madrid-away-kid-replica-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-grey-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
@@ -1477,25 +1458,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RFS</t>
+          <t>CFS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-09-26 08:53</t>
+          <t>2026-09-26 01:30</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>104055</v>
+        <v>81726</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>RFS_AH_HO_AD_No_26/27</t>
+          <t>CFS_NC_GreyGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Al Hilal Home Men Replica Football Shirt 2026/27</t>
+          <t>Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1505,23 +1486,27 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 68 ký tự (nên &lt;= 60)</t>
+          <t>khoảng trắng trước dấu câu: "Get the Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://replicafootballshirt.com/product/al-hilal-home-men-replica-football-shirt-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-grey-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
@@ -1543,20 +1528,20 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-09-26 01:30</t>
+          <t>2026-09-26 01:35</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>81726</v>
+        <v>81734</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CFS_NC_GreyGK_ADK_No_26/27</t>
+          <t>CFS_CHE_BlackGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1571,7 +1556,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 180 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1582,7 +1567,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/newcastle-united-grey-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -1604,20 +1589,20 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-09-26 01:30</t>
+          <t>2026-09-26 01:35</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>81726</v>
+        <v>81734</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CFS_NC_GreyGK_ADK_No_26/27</t>
+          <t>CFS_CHE_BlackGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1632,7 +1617,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Newcastle United Grey Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1647,7 +1632,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/newcastle-united-grey-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/chelsea-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
@@ -1669,20 +1654,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-26 01:35</t>
+          <t>2026-09-26 01:45</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>81734</v>
+        <v>81744</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CFS_CHE_BlackGK_ADK_No_26/27</t>
+          <t>CFS_AV_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1697,7 +1682,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 172 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1708,7 +1693,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/aston-villa-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
@@ -1730,20 +1715,20 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-09-26 01:35</t>
+          <t>2026-09-26 01:45</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>81734</v>
+        <v>81744</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CFS_CHE_BlackGK_ADK_No_26/27</t>
+          <t>CFS_AV_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1758,7 +1743,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Chelsea Black Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1773,7 +1758,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/chelsea-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/aston-villa-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
@@ -1795,20 +1780,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-09-26 01:45</t>
+          <t>2026-09-26 13:11</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>81744</v>
+        <v>81765</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CFS_AV_GreenGK_ADK_No_26/27</t>
+          <t>CFS_Ajax_BlackGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1823,7 +1808,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1834,7 +1819,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/aston-villa-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/ajax-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
@@ -1856,20 +1841,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-09-26 01:45</t>
+          <t>2026-09-26 13:11</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>81744</v>
+        <v>81765</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CFS_AV_GreenGK_ADK_No_26/27</t>
+          <t>CFS_Ajax_BlackGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1884,7 +1869,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Aston Villa Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -1899,7 +1884,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/aston-villa-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/ajax-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -1921,20 +1906,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-09-26 13:11</t>
+          <t>2026-09-26 13:17</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>81765</v>
+        <v>81776</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CFS_Ajax_BlackGK_ADK_No_26/27</t>
+          <t>CFS_Ajax_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1960,7 +1945,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/ajax-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/ajax-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
@@ -1982,20 +1967,20 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-09-26 13:11</t>
+          <t>2026-09-26 13:17</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>81765</v>
+        <v>81776</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CFS_Ajax_BlackGK_ADK_No_26/27</t>
+          <t>CFS_Ajax_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2010,7 +1995,7 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Ajax Black Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -2025,7 +2010,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/ajax-black-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/ajax-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -2047,20 +2032,20 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-09-26 13:17</t>
+          <t>2026-09-26 13:27</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>81776</v>
+        <v>81796</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CFS_Ajax_GreenGK_ADK_No_26/27</t>
+          <t>CFS_NC_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2070,12 +2055,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Meta description</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 169 ký tự (nên &lt;= 160)</t>
+          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -2086,7 +2071,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/ajax-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
@@ -2108,20 +2093,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-09-26 13:17</t>
+          <t>2026-09-26 13:27</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>81776</v>
+        <v>81796</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CFS_Ajax_GreenGK_ADK_No_26/27</t>
+          <t>CFS_NC_GreenGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2136,22 +2121,18 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Ajax Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>Meta dài 181 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Sửa định dạng</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/ajax-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -2196,20 +2177,24 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Meta description</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
+          <t>khoảng trắng trước dấu câu: "Get the Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
@@ -2234,20 +2219,20 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-09-26 13:27</t>
+          <t>2026-09-26 13:37</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>81796</v>
+        <v>81814</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CFS_NC_GreenGK_ADK_No_26/27</t>
+          <t>CFS_ITM_YellowGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2262,7 +2247,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 181 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 177 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -2273,7 +2258,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
@@ -2295,20 +2280,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-09-26 13:27</t>
+          <t>2026-09-26 13:37</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>81796</v>
+        <v>81814</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CFS_NC_GreenGK_ADK_No_26/27</t>
+          <t>CFS_ITM_YellowGK_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2323,7 +2308,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Newcastle United Green Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -2338,7 +2323,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/newcastle-united-green-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -2360,20 +2345,20 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-09-26 13:37</t>
+          <t>2026-09-26 13:46</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>81814</v>
+        <v>81825</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CFS_ITM_YellowGK_ADK_No_26/27</t>
+          <t>CFS_ITM_YellowGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2388,7 +2373,7 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 177 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -2399,7 +2384,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -2421,20 +2406,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-09-26 13:37</t>
+          <t>2026-09-26 13:46</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>81814</v>
+        <v>81825</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CFS_ITM_YellowGK_ADK_No_26/27</t>
+          <t>CFS_ITM_YellowGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27</t>
+          <t>Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2449,7 +2434,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Inter Milan Yellow Goalkeeper Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>khoảng trắng trước dấu câu: "Get the Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -2464,7 +2449,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
@@ -2486,20 +2471,20 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-09-26 13:46</t>
+          <t>2026-09-26 13:52</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>81825</v>
+        <v>81836</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CFS_ITM_YellowGK_KD_No_26/27</t>
+          <t>CFS_RS_AW_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Real Sociedad Away Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2514,7 +2499,7 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 176 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 173 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2525,7 +2510,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/real-sociedad-away-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -2547,20 +2532,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-09-26 13:46</t>
+          <t>2026-09-26 13:58</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>81825</v>
+        <v>81845</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CFS_ITM_YellowGK_KD_No_26/27</t>
+          <t>CFS_RS_HO_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27</t>
+          <t>Real Sociedad Home Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2575,22 +2560,18 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Inter Milan Yellow Goalkeeper Kids Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>Meta dài 173 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Sửa định dạng</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-yellow-goalkeeper-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/real-sociedad-home-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
@@ -2612,20 +2593,20 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-09-26 13:52</t>
+          <t>2026-09-26 14:11</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>81836</v>
+        <v>81863</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CFS_RS_AW_ADK_No_26/27</t>
+          <t>CFS_MC_AW_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Real Sociedad Away Adult Cheap Football Kit 2026/27</t>
+          <t>Manchester City Away Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2640,7 +2621,7 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 173 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 168 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2651,7 +2632,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-sociedad-away-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/manchester-city-away-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
@@ -2673,20 +2654,20 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-09-26 13:58</t>
+          <t>2026-09-26 14:11</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>81845</v>
+        <v>81863</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CFS_RS_HO_ADK_No_26/27</t>
+          <t>CFS_MC_AW_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Real Sociedad Home Adult Cheap Football Kit 2026/27</t>
+          <t>Manchester City Away Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2701,18 +2682,22 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 173 ký tự (nên &lt;= 160)</t>
+          <t>khoảng trắng trước dấu câu: "Get the Manchester City Away Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
+          <t>Sửa định dạng</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/real-sociedad-home-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/manchester-city-away-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M31" s="6" t="inlineStr">
@@ -2734,20 +2719,20 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-09-26 14:11</t>
+          <t>2026-09-26 14:21</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>81863</v>
+        <v>81874</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CFS_MC_AW_ADK_No_26/27</t>
+          <t>CFS_NAP_HO_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Manchester City Away Adult Cheap Football Kit 2026/27</t>
+          <t>SSC Napoli Home Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2762,7 +2747,7 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Meta dài 168 ký tự (nên &lt;= 160)</t>
+          <t>Meta dài 170 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2773,7 +2758,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/manchester-city-away-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/ssc-napoli-home-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
@@ -2795,20 +2780,20 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-09-26 14:11</t>
+          <t>2026-09-26 14:35</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>81863</v>
+        <v>81885</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CFS_MC_AW_ADK_No_26/27</t>
+          <t>CFS_EVE_HO_ADK_No_26/27</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Manchester City Away Adult Cheap Football Kit 2026/27</t>
+          <t>Everton Home Adult Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2823,22 +2808,18 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>khoảng trắng trước dấu câu: "Get the Manchester City Away Adult Cheap Football Kit 2026/27 , High Quality, Discounted Price, Risk-Free Shopping, Quick Support. Order now at Cheap Football Shirts ⚽️"</t>
+          <t>Meta dài 167 ký tự (nên &lt;= 160)</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Sửa định dạng</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
+          <t>Rút gọn</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/manchester-city-away-adult-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/everton-home-adult-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="M33" s="6" t="inlineStr">
@@ -2847,130 +2828,8 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>CFS</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2026-09-26 14:21</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>81874</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>CFS_NAP_HO_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>SSC Napoli Home Adult Cheap Football Kit 2026/27</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Meta description</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>Meta dài 170 ký tự (nên &lt;= 160)</t>
-        </is>
-      </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/ssc-napoli-home-adult-cheap-football-kit-2026-27/</t>
-        </is>
-      </c>
-      <c r="M34" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>Thấp</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CFS</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2026-09-26 14:35</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>81885</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>CFS_EVE_HO_ADK_No_26/27</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Everton Home Adult Cheap Football Kit 2026/27</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>SEO</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Meta description</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>Meta dài 167 ký tự (nên &lt;= 160)</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>Rút gọn</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>https://cheapfootballshirts.com/product/everton-home-adult-cheap-football-kit-2026-27/</t>
-        </is>
-      </c>
-      <c r="M35" s="6" t="inlineStr">
-        <is>
-          <t>Mở</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M35"/>
+  <autoFilter ref="A1:M33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3036,10 +2895,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3051,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3073,84 +2928,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Short sleeve</t>
+          <t>Trustpilot / 4.9★</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>SOP: không bao giờ nhắc short sleeve. Description KFK (130/162 listing), RFK (107/289), CFS (6) đang có 'Short-Sleeve shirt' / 'short sleeves'. Có cần xoá không?</t>
+          <t>SOP: tránh 'Trustpilot' và claim 4.9★. Short description KFK, RFS, RFK có dòng 'Rated 4.9 on Trustpilot' (CFS không có). Giữ hay bỏ?</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Trustpilot / 4.9★</t>
+          <t>Tên né thương hiệu</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>SOP: tránh 'Trustpilot' và claim 4.9★. Short description KFK, RFS, RFK có dòng 'Rated 4.9 on Trustpilot' (CFS không có). Giữ hay bỏ?</t>
+          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG và nhận ra kiểu 'Arsn@l', 'Lvr^_^pooI'.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tên né thương hiệu</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Tool coi 'North London Red' = Arsenal, 'P^_^SG' = PSG và nhận ra kiểu 'Arsn@l', 'Lvr^_^pooI'.</t>
+          <t>Tool KHÔNG báo lỗi 'sleeve badge' (tên option), chỉ báo 'badge' đứng riêng.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sleeve badge</t>
+          <t>Độ dài SEO title</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tool KHÔNG báo lỗi 'sleeve badge' (tên option), chỉ báo 'badge' đứng riêng.</t>
+          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Độ dài SEO title</t>
+          <t>KFK / CFS / RFK template SEO</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Tool báo khi SEO title &gt; 65 ký tự và meta &gt; 165 ký tự (mức Thấp).</t>
+          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KFK / CFS / RFK template SEO</t>
+          <t>Đã xác nhận 27/9</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>SOP chưa có template SEO title/meta cho KFK, CFS, RFK nên tool chưa check đúng mẫu cho các site này, chỉ check nội dung có khớp sản phẩm không.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Đã xác nhận 27/9</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>ADK = Adult Kit. Gift pack noindex là cố ý (không báo lỗi). Listing in 'CHAMPIONS 26 / WINNERS 26' không cần player attribute.</t>
+          <t>ADK = Adult Kit. Gift pack noindex là cố ý (không báo lỗi). Listing in 'CHAMPIONS 26 / WINNERS 26' không cần player attribute. Nhắc 'short sleeve' được, chỉ báo khi mâu thuẫn với Long Sleeve (tên/SKU/ảnh).</t>
         </is>
       </c>
     </row>

</xml_diff>